<commit_message>
Finish the four partial Time LOM fixtures with Kyle identities.
33612-1, 105098-1, 103516 (+ nested 103535-1), and 1004611-1 now assert the full (part_no, qty) set. Empty 103535-1 tab still fails as an empty L2 shell. S 80054-1 gasket qty is 10 inches, not 10 pieces. Zero partials remain.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/lom/103516-LOM.xlsx
+++ b/tests/fixtures/lom/103516-LOM.xlsx
@@ -74,7 +74,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -84,7 +84,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t/>
+          <t>103541-1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -101,7 +101,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -111,7 +111,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t/>
+          <t>103540-1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -128,7 +128,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -138,7 +138,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t/>
+          <t>103539-1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -155,7 +155,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -165,7 +165,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t/>
+          <t>103538-1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -182,7 +182,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -192,7 +192,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t/>
+          <t>103537-1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -209,7 +209,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -219,7 +219,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t/>
+          <t>103536-1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -263,7 +263,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t/>
+          <t>30345-19</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -290,7 +290,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -300,7 +300,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t/>
+          <t>103534-1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -317,7 +317,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -327,7 +327,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t/>
+          <t>103533-1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -344,7 +344,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -354,7 +354,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t/>
+          <t>103532-1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -371,7 +371,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -381,7 +381,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t/>
+          <t>103531-1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -398,7 +398,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -408,7 +408,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t/>
+          <t>103530-1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -425,7 +425,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -435,7 +435,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t/>
+          <t>103529-1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -452,7 +452,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t/>
+          <t>103528-1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t/>
+          <t>103527-1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t/>
+          <t>103526-1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t/>
+          <t>103525-1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t/>
+          <t>103524-1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t/>
+          <t>103523-1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t/>
+          <t>103522-1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t/>
+          <t>103521-1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t/>
+          <t>103520-1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t/>
+          <t>103519-1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t/>
+          <t>103518-1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t/>
+          <t>103517-1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -778,7 +778,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>QTY</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -794,6 +794,204 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>103546-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GATE STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>671700</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HINGE SELF CLOSING 1-PAIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>102196-5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PLATE (HINGE PLATE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>103545-1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GATE GUSSET</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>101229-4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BAR ROUND 1/2 DIA.(STRIKER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>30345-20</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PLATE (STRIKER BRACE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>103544-1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>STRIKER MOUNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>103543-1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GATE RAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>103542-1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GATE RAIL</t>
         </is>
       </c>
     </row>
@@ -851,22 +1049,572 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>103541-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>103540-1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>103539-1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>103538-1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>103537-1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>103536-1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>103535-1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>GATE WELDMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30345-19</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>103534-1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>103533-1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>103532-1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>103531-1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>103530-1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>103529-1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>103528-1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>103527-1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>103526-1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>103525-1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>103524-1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>103523-1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>103522-1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>103521-1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>103520-1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>103519-1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>103518-1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>103517-1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>